<commit_message>
updated zephyr in config
</commit_message>
<xml_diff>
--- a/target/test-classes/testdata.xlsx
+++ b/target/test-classes/testdata.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="162">
   <si>
     <t>PASS</t>
   </si>
@@ -429,6 +429,81 @@
   </si>
   <si>
     <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaLanguageSelector_TestNG-test-WebRegressionSuite-1_20261012_122917_721.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 13:47:56</t>
+  </si>
+  <si>
+    <t>2853</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaArticleSearch_TestNG-test-WebRegressionSuite-3_20261012_134756_735.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 13:47:58</t>
+  </si>
+  <si>
+    <t>1042</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumHeroSection_TestNG-test-WebRegressionSuite-3_20261012_134758_860.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 13:48:01</t>
+  </si>
+  <si>
+    <t>1046</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDocumentationPage_TestNG-test-WebRegressionSuite-3_20261012_134801_051.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 13:48:02</t>
+  </si>
+  <si>
+    <t>613</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 13:48:04</t>
+  </si>
+  <si>
+    <t>524</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 13:48:06</t>
+  </si>
+  <si>
+    <t>917</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaPortalTaglineInTitle_TestNG-test-WebRegressionSuite-3_20261012_134806_487.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 13:48:11</t>
+  </si>
+  <si>
+    <t>2033</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDownloadsPageTitle_TestNG-test-WebRegressionSuite-3_20261012_134811_223.png</t>
+  </si>
+  <si>
+    <t>15825</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 13:48:28</t>
+  </si>
+  <si>
+    <t>15583</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 13:48:44</t>
+  </si>
+  <si>
+    <t>15588</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaLanguageSelector_TestNG-test-WebRegressionSuite-1_20261012_134844_857.png</t>
   </si>
 </sst>
 </file>
@@ -959,13 +1034,13 @@
         <v>PASS</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
-        <v>12-Oct-2026 12:28:26</v>
+        <v>12-Oct-2026 13:47:54</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
-        <v>3792</v>
+        <v>3260</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
-        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyAmazonHomePageTitle_TestNG-test-WebRegressionSuite-1_20261012_122826_748.png</v>
+        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyAmazonHomePageTitle_TestNG-test-WebRegressionSuite-1_20261012_134754_342.png</v>
       </c>
     </row>
     <row r="3">
@@ -998,13 +1073,13 @@
         <v>PASS</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
-        <v>12-Oct-2026 12:28:44</v>
+        <v>12-Oct-2026 13:48:10</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
-        <v>21706</v>
+        <v>19822</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
-        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyFlipkartHomePageTitle_TestNG-test-WebRegressionSuite-2_20261012_122844_572.png</v>
+        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyFlipkartHomePageTitle_TestNG-test-WebRegressionSuite-2_20261012_134810_516.png</v>
       </c>
     </row>
     <row r="4">
@@ -1037,13 +1112,13 @@
         <v>PASS</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
-        <v>12-Oct-2026 12:28:24</v>
+        <v>12-Oct-2026 13:47:51</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
-        <v>1574</v>
+        <v>1586</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
-        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaHomePageTitle_TestNG-test-WebRegressionSuite-3_20261012_122824_006.png</v>
+        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaHomePageTitle_TestNG-test-WebRegressionSuite-3_20261012_134751_711.png</v>
       </c>
     </row>
     <row r="5">
@@ -1076,13 +1151,13 @@
         <v>PASS</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
-        <v>12-Oct-2026 12:28:40</v>
+        <v>12-Oct-2026 13:48:07</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
-        <v>18100</v>
+        <v>17495</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
-        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumHomePageTitle_TestNG-test-WebRegressionSuite-4_20261012_122840_573.png</v>
+        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumHomePageTitle_TestNG-test-WebRegressionSuite-4_20261012_134807_817.png</v>
       </c>
     </row>
     <row r="6">
@@ -1115,13 +1190,13 @@
         <v>0</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>111</v>
+        <v>137</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>112</v>
+        <v>138</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>113</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7">
@@ -1154,13 +1229,13 @@
         <v>22</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>134</v>
+        <v>159</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8">
@@ -1193,13 +1268,13 @@
         <v>0</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>114</v>
+        <v>140</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>115</v>
+        <v>141</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>116</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9">
@@ -1232,13 +1307,13 @@
         <v>0</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>117</v>
+        <v>143</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>118</v>
+        <v>144</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>119</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10">
@@ -1271,13 +1346,13 @@
         <v>22</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>125</v>
+        <v>151</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>126</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11">
@@ -1310,13 +1385,13 @@
         <v>0</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>128</v>
+        <v>154</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>129</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>